<commit_message>
add randomise & plots
</commit_message>
<xml_diff>
--- a/code/SFNCovariatesSubList.xlsx
+++ b/code/SFNCovariatesSubList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswyngaarden/Documents/GitHub/rf1-sra-socdoors/code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6184BF09-DB11-5B4B-A8A0-D495EE59485C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9503301C-D8DC-7644-81BF-514C5B7A849A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16540" activeTab="4" xr2:uid="{E21B9450-44FE-AB4C-A453-866E41E6C653}"/>
+    <workbookView xWindow="10020" yWindow="500" windowWidth="18780" windowHeight="16580" xr2:uid="{E21B9450-44FE-AB4C-A453-866E41E6C653}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="ageXnbs" sheetId="3" r:id="rId3"/>
     <sheet name="ageXoafem" sheetId="4" r:id="rId4"/>
     <sheet name="ageXnbsXoafem" sheetId="5" r:id="rId5"/>
+    <sheet name="ageXmspss" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="165">
   <si>
     <t>tania_subid</t>
   </si>
@@ -527,6 +528,15 @@
   <si>
     <t>nbs*oafem</t>
   </si>
+  <si>
+    <t>mspss</t>
+  </si>
+  <si>
+    <t>ageXmspss</t>
+  </si>
+  <si>
+    <t>RM:</t>
+  </si>
 </sst>
 </file>
 
@@ -564,11 +574,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -883,7 +891,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{912C04A1-F94E-4949-B87C-4FFD46883FA1}">
-  <dimension ref="A1:ES60"/>
+  <dimension ref="A1:ES63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="93" max="93" width="10.83203125" style="1" customWidth="1"/>
@@ -3565,32 +3573,32 @@
         <v>133</v>
       </c>
     </row>
-    <row r="7" spans="1:149" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+    <row r="7" spans="1:149" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>10486</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>41.91</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
         <v>-1.1424137931034508</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7">
         <v>3</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
         <v>-7.9310344827586032E-2</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7">
         <v>19</v>
       </c>
       <c r="G7">
         <f t="shared" si="2"/>
         <v>11.568965517241379</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" t="s">
         <v>133</v>
       </c>
       <c r="I7">
@@ -3609,406 +3617,406 @@
         <f t="shared" si="6"/>
         <v>1.0482088031489605</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7">
         <v>131381</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7">
         <v>5.6666670000000003</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7">
         <v>6</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7">
         <v>5</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7">
         <v>6.5714290000000002</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7">
         <v>6.8571429999999998</v>
       </c>
-      <c r="S7" s="2">
+      <c r="S7">
         <v>4.6666670000000003</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="T7" t="s">
         <v>131</v>
       </c>
-      <c r="U7" s="2" t="s">
+      <c r="U7" t="s">
         <v>132</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7">
         <v>4.33</v>
       </c>
-      <c r="W7" s="2">
+      <c r="W7">
         <v>3.9</v>
       </c>
-      <c r="X7" s="2">
+      <c r="X7">
         <v>4</v>
       </c>
-      <c r="Y7" s="2">
+      <c r="Y7">
         <v>4</v>
       </c>
-      <c r="Z7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="2">
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
         <v>4.33</v>
       </c>
-      <c r="AB7" s="2">
+      <c r="AB7">
         <v>3.83</v>
       </c>
-      <c r="AC7" s="2">
+      <c r="AC7">
         <v>4.63</v>
       </c>
-      <c r="AD7" s="2">
+      <c r="AD7">
         <v>4.17</v>
       </c>
-      <c r="AE7" s="2">
+      <c r="AE7">
         <v>4.4000000000000004</v>
       </c>
-      <c r="AF7" s="2">
+      <c r="AF7">
         <v>37</v>
       </c>
-      <c r="AG7" s="2">
+      <c r="AG7">
         <v>9</v>
       </c>
-      <c r="AH7" s="2">
+      <c r="AH7">
         <v>15</v>
       </c>
-      <c r="AI7" s="2">
+      <c r="AI7">
         <v>6</v>
       </c>
-      <c r="AJ7" s="2">
+      <c r="AJ7">
         <v>7</v>
       </c>
-      <c r="AK7" s="2">
+      <c r="AK7">
         <v>3</v>
       </c>
-      <c r="AL7" s="2">
+      <c r="AL7">
         <v>7</v>
       </c>
-      <c r="AM7" s="2">
+      <c r="AM7">
         <v>5</v>
       </c>
-      <c r="AN7" s="2">
+      <c r="AN7">
         <v>6</v>
       </c>
-      <c r="AO7" s="2">
+      <c r="AO7">
         <v>2</v>
       </c>
-      <c r="AP7" s="2">
+      <c r="AP7">
         <v>23</v>
       </c>
-      <c r="AQ7" s="2">
+      <c r="AQ7">
         <v>35</v>
       </c>
-      <c r="AR7" s="2">
+      <c r="AR7">
         <v>14</v>
       </c>
-      <c r="AS7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AT7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AU7" s="2">
+      <c r="AS7">
+        <v>0</v>
+      </c>
+      <c r="AT7">
+        <v>0</v>
+      </c>
+      <c r="AU7">
         <v>4.75</v>
       </c>
-      <c r="AV7" s="2">
+      <c r="AV7">
         <v>5.25</v>
       </c>
-      <c r="AW7" s="2">
+      <c r="AW7">
         <v>5</v>
       </c>
-      <c r="AX7" s="2">
+      <c r="AX7">
         <v>4</v>
       </c>
-      <c r="AZ7" s="2">
+      <c r="AZ7">
         <v>15</v>
       </c>
-      <c r="BA7" s="2">
+      <c r="BA7">
         <v>3.08</v>
       </c>
-      <c r="BC7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BD7" s="2">
+      <c r="BC7">
+        <v>0</v>
+      </c>
+      <c r="BD7">
         <v>3.51</v>
       </c>
-      <c r="BE7" s="2">
+      <c r="BE7">
         <v>29</v>
       </c>
-      <c r="BF7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BG7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BH7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BI7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BJ7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BK7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BL7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BM7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BN7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BO7" s="2">
+      <c r="BF7">
+        <v>0</v>
+      </c>
+      <c r="BG7">
+        <v>0</v>
+      </c>
+      <c r="BH7">
+        <v>0</v>
+      </c>
+      <c r="BI7">
+        <v>0</v>
+      </c>
+      <c r="BJ7">
+        <v>0</v>
+      </c>
+      <c r="BK7">
+        <v>0</v>
+      </c>
+      <c r="BL7">
+        <v>0</v>
+      </c>
+      <c r="BM7">
+        <v>0</v>
+      </c>
+      <c r="BN7">
+        <v>0</v>
+      </c>
+      <c r="BO7">
         <v>20</v>
       </c>
-      <c r="BP7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BQ7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BR7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BS7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BT7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BU7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BV7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BW7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BX7" s="2">
+      <c r="BP7">
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <v>0</v>
+      </c>
+      <c r="BR7">
+        <v>0</v>
+      </c>
+      <c r="BS7">
+        <v>0</v>
+      </c>
+      <c r="BT7">
+        <v>0</v>
+      </c>
+      <c r="BU7">
+        <v>0</v>
+      </c>
+      <c r="BV7">
+        <v>0</v>
+      </c>
+      <c r="BW7">
+        <v>0</v>
+      </c>
+      <c r="BX7">
         <v>8991</v>
       </c>
-      <c r="BY7" s="2">
-        <v>0</v>
-      </c>
-      <c r="BZ7" s="2">
-        <v>0</v>
-      </c>
-      <c r="CA7" s="2">
-        <v>0</v>
-      </c>
-      <c r="CB7" s="2">
-        <v>0</v>
-      </c>
-      <c r="CC7" s="2">
+      <c r="BY7">
+        <v>0</v>
+      </c>
+      <c r="BZ7">
+        <v>0</v>
+      </c>
+      <c r="CA7">
+        <v>0</v>
+      </c>
+      <c r="CB7">
+        <v>0</v>
+      </c>
+      <c r="CC7">
         <v>3.7</v>
       </c>
-      <c r="CD7" s="2">
+      <c r="CD7">
         <v>3.9</v>
       </c>
-      <c r="CE7" s="2">
+      <c r="CE7">
         <v>3.9</v>
       </c>
-      <c r="CF7" s="2">
+      <c r="CF7">
         <v>3.83</v>
       </c>
-      <c r="CG7" s="2">
+      <c r="CG7">
         <v>6</v>
       </c>
-      <c r="CH7" s="2">
+      <c r="CH7">
         <v>4.3333333333333304</v>
       </c>
-      <c r="CI7" s="2">
+      <c r="CI7">
         <v>2.6666666666666599</v>
       </c>
-      <c r="CJ7" s="2">
+      <c r="CJ7">
         <v>1.8333333333333299</v>
       </c>
-      <c r="CK7" s="2">
+      <c r="CK7">
         <v>2.95</v>
       </c>
-      <c r="CL7" s="2">
-        <v>0</v>
-      </c>
-      <c r="CM7" s="2">
-        <v>0</v>
-      </c>
-      <c r="CN7" s="2">
+      <c r="CL7">
+        <v>0</v>
+      </c>
+      <c r="CM7">
+        <v>0</v>
+      </c>
+      <c r="CN7">
         <v>27</v>
       </c>
-      <c r="CO7" s="2">
+      <c r="CO7">
         <v>24</v>
       </c>
-      <c r="CP7" s="2">
+      <c r="CP7">
         <v>11</v>
       </c>
-      <c r="CQ7" s="2">
+      <c r="CQ7">
         <v>1.1000000000000001</v>
       </c>
-      <c r="CR7" s="2">
+      <c r="CR7">
         <v>38</v>
       </c>
-      <c r="CS7" s="2">
+      <c r="CS7">
         <v>40</v>
       </c>
-      <c r="CT7" s="2">
+      <c r="CT7">
         <v>39</v>
       </c>
-      <c r="CU7" s="3">
+      <c r="CU7" s="1">
         <v>23</v>
       </c>
-      <c r="CV7" s="3">
+      <c r="CV7" s="1">
         <v>36</v>
       </c>
-      <c r="CW7" s="2">
+      <c r="CW7">
         <v>47</v>
       </c>
-      <c r="CX7" s="2">
-        <v>0</v>
-      </c>
-      <c r="CY7" s="2">
+      <c r="CX7">
+        <v>0</v>
+      </c>
+      <c r="CY7">
         <v>47</v>
       </c>
-      <c r="CZ7" s="2">
+      <c r="CZ7">
         <v>60</v>
       </c>
-      <c r="DA7" s="2">
+      <c r="DA7">
         <v>34</v>
       </c>
-      <c r="DB7" s="2">
+      <c r="DB7">
         <v>60</v>
       </c>
-      <c r="DC7" s="2">
-        <v>0</v>
-      </c>
-      <c r="DD7" s="2">
-        <v>0</v>
-      </c>
-      <c r="DE7" s="2">
+      <c r="DC7">
+        <v>0</v>
+      </c>
+      <c r="DD7">
+        <v>0</v>
+      </c>
+      <c r="DE7">
         <v>4</v>
       </c>
-      <c r="DF7" s="2">
+      <c r="DF7">
         <v>4</v>
       </c>
-      <c r="DG7" s="2">
+      <c r="DG7">
         <v>45105</v>
       </c>
-      <c r="DH7" s="2">
+      <c r="DH7">
         <v>29682</v>
       </c>
-      <c r="DI7" s="2">
+      <c r="DI7">
         <v>42.23</v>
       </c>
-      <c r="DJ7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DK7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DL7" s="2">
-        <v>1</v>
-      </c>
-      <c r="DM7" s="2">
-        <v>0</v>
-      </c>
-      <c r="DN7" s="2">
-        <v>1</v>
-      </c>
-      <c r="DO7" s="2">
+      <c r="DJ7" t="s">
+        <v>133</v>
+      </c>
+      <c r="DK7" t="s">
+        <v>133</v>
+      </c>
+      <c r="DL7">
+        <v>1</v>
+      </c>
+      <c r="DM7">
+        <v>0</v>
+      </c>
+      <c r="DN7">
+        <v>1</v>
+      </c>
+      <c r="DO7">
         <v>5</v>
       </c>
-      <c r="DP7" s="2">
+      <c r="DP7">
         <v>23</v>
       </c>
-      <c r="DQ7" s="2">
+      <c r="DQ7">
         <v>2.1111111111111001</v>
       </c>
-      <c r="DR7" s="2">
+      <c r="DR7">
         <v>9</v>
       </c>
-      <c r="DS7" s="2">
+      <c r="DS7">
         <v>999</v>
       </c>
-      <c r="DT7" s="2">
+      <c r="DT7">
         <v>5</v>
       </c>
-      <c r="DU7" s="2">
+      <c r="DU7">
         <v>2</v>
       </c>
-      <c r="DV7" s="2">
+      <c r="DV7">
         <v>999</v>
       </c>
-      <c r="DW7" s="2">
+      <c r="DW7">
         <v>9</v>
       </c>
-      <c r="DY7" s="2">
+      <c r="DY7">
         <v>6</v>
       </c>
-      <c r="DZ7" s="2">
+      <c r="DZ7">
         <v>2</v>
       </c>
-      <c r="EA7" s="2">
+      <c r="EA7">
         <v>6</v>
       </c>
-      <c r="EB7" s="2">
+      <c r="EB7">
         <v>6</v>
       </c>
-      <c r="EC7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ED7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EE7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EF7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EG7" s="2">
+      <c r="EC7" t="s">
+        <v>133</v>
+      </c>
+      <c r="ED7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EE7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EF7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EG7">
         <v>19403</v>
       </c>
-      <c r="EH7" s="2">
+      <c r="EH7">
         <v>6</v>
       </c>
-      <c r="EI7" s="2">
-        <v>1</v>
-      </c>
-      <c r="EJ7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EK7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EL7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EM7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EN7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EO7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EP7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EQ7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ER7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ES7" s="2" t="s">
+      <c r="EI7">
+        <v>1</v>
+      </c>
+      <c r="EJ7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EK7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EL7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EM7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EN7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EO7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EP7" t="s">
+        <v>133</v>
+      </c>
+      <c r="EQ7" t="s">
+        <v>133</v>
+      </c>
+      <c r="ER7" t="s">
+        <v>133</v>
+      </c>
+      <c r="ES7" t="s">
         <v>133</v>
       </c>
     </row>
@@ -4906,32 +4914,32 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:149" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+    <row r="10" spans="1:149" x14ac:dyDescent="0.2">
+      <c r="A10">
         <v>10572</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
         <v>70.459999999999994</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
         <v>27.407586206896546</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10">
         <v>2.6</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
         <v>-0.47931034482758594</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
         <f t="shared" si="2"/>
         <v>-7.431034482758621</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" t="s">
         <v>133</v>
       </c>
       <c r="I10">
@@ -4950,406 +4958,406 @@
         <f t="shared" si="6"/>
         <v>97.619564926811194</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10">
         <v>10252</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10">
         <v>3</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10">
         <v>3.0909089999999999</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10">
         <v>3.5</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10">
         <v>3.454545</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10">
         <v>4.5454549999999996</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10">
         <v>3.1666669999999999</v>
       </c>
-      <c r="T10" s="2" t="s">
+      <c r="T10" t="s">
         <v>131</v>
       </c>
-      <c r="U10" s="2" t="s">
+      <c r="U10" t="s">
         <v>132</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10">
         <v>4.22</v>
       </c>
-      <c r="W10" s="2">
+      <c r="W10">
         <v>3.1</v>
       </c>
-      <c r="X10" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="2">
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
         <v>6.17</v>
       </c>
-      <c r="AB10" s="2">
+      <c r="AB10">
         <v>5.67</v>
       </c>
-      <c r="AC10" s="2">
+      <c r="AC10">
         <v>6.13</v>
       </c>
-      <c r="AD10" s="2">
+      <c r="AD10">
         <v>5.17</v>
       </c>
-      <c r="AE10" s="2">
+      <c r="AE10">
         <v>5.83</v>
       </c>
-      <c r="AF10" s="2">
+      <c r="AF10">
         <v>4</v>
       </c>
-      <c r="AG10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH10" s="2">
-        <v>1</v>
-      </c>
-      <c r="AI10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AJ10" s="2">
+      <c r="AG10">
+        <v>0</v>
+      </c>
+      <c r="AH10">
+        <v>1</v>
+      </c>
+      <c r="AI10">
+        <v>0</v>
+      </c>
+      <c r="AJ10">
         <v>3</v>
       </c>
-      <c r="AK10" s="2">
+      <c r="AK10">
         <v>2</v>
       </c>
-      <c r="AL10" s="2">
+      <c r="AL10">
         <v>4</v>
       </c>
-      <c r="AM10" s="2">
+      <c r="AM10">
         <v>5</v>
       </c>
-      <c r="AN10" s="2">
+      <c r="AN10">
         <v>3</v>
       </c>
-      <c r="AO10" s="2">
+      <c r="AO10">
         <v>4</v>
       </c>
-      <c r="AP10" s="2">
+      <c r="AP10">
         <v>18</v>
       </c>
-      <c r="AQ10" s="2">
+      <c r="AQ10">
         <v>31</v>
       </c>
-      <c r="AR10" s="2">
+      <c r="AR10">
         <v>12</v>
       </c>
-      <c r="AS10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AT10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AU10" s="2">
+      <c r="AS10">
+        <v>0</v>
+      </c>
+      <c r="AT10">
+        <v>0</v>
+      </c>
+      <c r="AU10">
         <v>6</v>
       </c>
-      <c r="AV10" s="2">
+      <c r="AV10">
         <v>6</v>
       </c>
-      <c r="AW10" s="2">
+      <c r="AW10">
         <v>6</v>
       </c>
-      <c r="AX10" s="2">
+      <c r="AX10">
         <v>6</v>
       </c>
-      <c r="AZ10" s="2">
+      <c r="AZ10">
         <v>6</v>
       </c>
-      <c r="BA10" s="2">
+      <c r="BA10">
         <v>2.25</v>
       </c>
-      <c r="BC10" s="2">
+      <c r="BC10">
         <v>3.17</v>
       </c>
-      <c r="BD10" s="2">
+      <c r="BD10">
         <v>2.69</v>
       </c>
-      <c r="BE10" s="2">
+      <c r="BE10">
         <v>72</v>
       </c>
-      <c r="BF10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BG10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BH10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BI10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BJ10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BK10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BL10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BM10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BN10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BO10" s="2">
+      <c r="BF10">
+        <v>0</v>
+      </c>
+      <c r="BG10">
+        <v>0</v>
+      </c>
+      <c r="BH10">
+        <v>0</v>
+      </c>
+      <c r="BI10">
+        <v>0</v>
+      </c>
+      <c r="BJ10">
+        <v>0</v>
+      </c>
+      <c r="BK10">
+        <v>0</v>
+      </c>
+      <c r="BL10">
+        <v>0</v>
+      </c>
+      <c r="BM10">
+        <v>0</v>
+      </c>
+      <c r="BN10">
+        <v>0</v>
+      </c>
+      <c r="BO10">
         <v>20</v>
       </c>
-      <c r="BP10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BQ10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BR10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BS10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BT10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BU10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BV10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BW10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BX10" s="2">
+      <c r="BP10">
+        <v>0</v>
+      </c>
+      <c r="BQ10">
+        <v>0</v>
+      </c>
+      <c r="BR10">
+        <v>0</v>
+      </c>
+      <c r="BS10">
+        <v>0</v>
+      </c>
+      <c r="BT10">
+        <v>0</v>
+      </c>
+      <c r="BU10">
+        <v>0</v>
+      </c>
+      <c r="BV10">
+        <v>0</v>
+      </c>
+      <c r="BW10">
+        <v>0</v>
+      </c>
+      <c r="BX10">
         <v>8991</v>
       </c>
-      <c r="BY10" s="2">
-        <v>0</v>
-      </c>
-      <c r="BZ10" s="2">
-        <v>0</v>
-      </c>
-      <c r="CA10" s="2">
-        <v>0</v>
-      </c>
-      <c r="CB10" s="2">
-        <v>0</v>
-      </c>
-      <c r="CC10" s="2">
+      <c r="BY10">
+        <v>0</v>
+      </c>
+      <c r="BZ10">
+        <v>0</v>
+      </c>
+      <c r="CA10">
+        <v>0</v>
+      </c>
+      <c r="CB10">
+        <v>0</v>
+      </c>
+      <c r="CC10">
         <v>3.2</v>
       </c>
-      <c r="CD10" s="2">
+      <c r="CD10">
         <v>3.3</v>
       </c>
-      <c r="CE10" s="2">
+      <c r="CE10">
         <v>3.7</v>
       </c>
-      <c r="CF10" s="2">
+      <c r="CF10">
         <v>3.4</v>
       </c>
-      <c r="CG10" s="2">
+      <c r="CG10">
         <v>2.6666666666666599</v>
       </c>
-      <c r="CH10" s="2">
+      <c r="CH10">
         <v>2.6666666666666599</v>
       </c>
-      <c r="CI10" s="2">
+      <c r="CI10">
         <v>4.3333333333333304</v>
       </c>
-      <c r="CJ10" s="2">
+      <c r="CJ10">
         <v>2.6666666666666599</v>
       </c>
-      <c r="CK10" s="2">
+      <c r="CK10">
         <v>0.3</v>
       </c>
-      <c r="CL10" s="2">
-        <v>0</v>
-      </c>
-      <c r="CM10" s="2">
-        <v>0</v>
-      </c>
-      <c r="CN10" s="2">
+      <c r="CL10">
+        <v>0</v>
+      </c>
+      <c r="CM10">
+        <v>0</v>
+      </c>
+      <c r="CN10">
         <v>29</v>
       </c>
-      <c r="CO10" s="2">
+      <c r="CO10">
         <v>18</v>
       </c>
-      <c r="CP10" s="2">
+      <c r="CP10">
         <v>11</v>
       </c>
-      <c r="CQ10" s="2">
+      <c r="CQ10">
         <v>0.91666666666666596</v>
       </c>
-      <c r="CR10" s="2">
+      <c r="CR10">
         <v>40</v>
       </c>
-      <c r="CS10" s="2">
+      <c r="CS10">
         <v>28</v>
       </c>
-      <c r="CT10" s="2">
+      <c r="CT10">
         <v>42</v>
       </c>
-      <c r="CU10" s="3">
+      <c r="CU10" s="1">
         <v>27</v>
       </c>
-      <c r="CV10" s="3">
+      <c r="CV10" s="1">
         <v>29</v>
       </c>
-      <c r="CW10" s="2">
+      <c r="CW10">
         <v>46</v>
       </c>
-      <c r="CX10" s="2">
+      <c r="CX10">
         <v>60</v>
       </c>
-      <c r="CY10" s="2">
+      <c r="CY10">
         <v>42</v>
       </c>
-      <c r="CZ10" s="2">
+      <c r="CZ10">
         <v>60</v>
       </c>
-      <c r="DA10" s="2">
+      <c r="DA10">
         <v>29</v>
       </c>
-      <c r="DB10" s="2">
+      <c r="DB10">
         <v>60</v>
       </c>
-      <c r="DC10" s="2">
-        <v>0</v>
-      </c>
-      <c r="DD10" s="2">
-        <v>0</v>
-      </c>
-      <c r="DE10" s="2">
+      <c r="DC10">
+        <v>0</v>
+      </c>
+      <c r="DD10">
+        <v>0</v>
+      </c>
+      <c r="DE10">
         <v>2</v>
       </c>
-      <c r="DF10" s="2">
-        <v>1</v>
-      </c>
-      <c r="DG10" s="2">
+      <c r="DF10">
+        <v>1</v>
+      </c>
+      <c r="DG10">
         <v>45106</v>
       </c>
-      <c r="DH10" s="2">
+      <c r="DH10">
         <v>19250</v>
       </c>
-      <c r="DI10" s="2">
+      <c r="DI10">
         <v>70.790000000000006</v>
       </c>
-      <c r="DJ10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DK10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DL10" s="2">
-        <v>1</v>
-      </c>
-      <c r="DM10" s="2">
-        <v>0</v>
-      </c>
-      <c r="DN10" s="2">
-        <v>0</v>
-      </c>
-      <c r="DO10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DP10" s="2">
+      <c r="DJ10" t="s">
+        <v>133</v>
+      </c>
+      <c r="DK10" t="s">
+        <v>133</v>
+      </c>
+      <c r="DL10">
+        <v>1</v>
+      </c>
+      <c r="DM10">
+        <v>0</v>
+      </c>
+      <c r="DN10">
+        <v>0</v>
+      </c>
+      <c r="DO10" t="s">
+        <v>133</v>
+      </c>
+      <c r="DP10">
         <v>28</v>
       </c>
-      <c r="DQ10" s="2">
+      <c r="DQ10">
         <v>2.3333333333333002</v>
       </c>
-      <c r="DR10" s="2">
+      <c r="DR10">
         <v>12</v>
       </c>
-      <c r="DS10" s="2">
+      <c r="DS10">
         <v>999</v>
       </c>
-      <c r="DT10" s="2">
+      <c r="DT10">
         <v>6</v>
       </c>
-      <c r="DU10" s="2">
+      <c r="DU10">
         <v>2</v>
       </c>
-      <c r="DV10" s="2">
+      <c r="DV10">
         <v>999</v>
       </c>
-      <c r="DW10" s="2">
+      <c r="DW10">
         <v>8</v>
       </c>
-      <c r="DY10" s="2">
+      <c r="DY10">
         <v>5</v>
       </c>
-      <c r="DZ10" s="2">
-        <v>1</v>
-      </c>
-      <c r="EA10" s="2">
+      <c r="DZ10">
+        <v>1</v>
+      </c>
+      <c r="EA10">
         <v>7</v>
       </c>
-      <c r="EB10" s="2">
+      <c r="EB10">
         <v>5</v>
       </c>
-      <c r="EC10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ED10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EE10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EF10" s="2">
-        <v>1</v>
-      </c>
-      <c r="EG10" s="2">
+      <c r="EC10" t="s">
+        <v>133</v>
+      </c>
+      <c r="ED10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EE10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EF10">
+        <v>1</v>
+      </c>
+      <c r="EG10">
         <v>18249</v>
       </c>
-      <c r="EH10" s="2">
+      <c r="EH10">
         <v>7</v>
       </c>
-      <c r="EI10" s="2">
-        <v>1</v>
-      </c>
-      <c r="EJ10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EK10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EL10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EM10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EN10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EO10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EP10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EQ10" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ER10" s="2">
-        <v>0</v>
-      </c>
-      <c r="ES10" s="2" t="s">
+      <c r="EI10">
+        <v>1</v>
+      </c>
+      <c r="EJ10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EK10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EL10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EM10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EN10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EO10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EP10" t="s">
+        <v>133</v>
+      </c>
+      <c r="EQ10" t="s">
+        <v>133</v>
+      </c>
+      <c r="ER10">
+        <v>0</v>
+      </c>
+      <c r="ES10" t="s">
         <v>133</v>
       </c>
     </row>
@@ -6247,32 +6255,32 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:149" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+    <row r="13" spans="1:149" x14ac:dyDescent="0.2">
+      <c r="A13">
         <v>10585</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <v>63.33</v>
       </c>
       <c r="C13">
         <f t="shared" si="0"/>
         <v>20.277586206896551</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13">
         <v>3</v>
       </c>
       <c r="E13">
         <f t="shared" si="1"/>
         <v>-7.9310344827586032E-2</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13">
         <v>8</v>
       </c>
       <c r="G13">
         <f t="shared" si="2"/>
         <v>0.568965517241379</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" t="s">
         <v>133</v>
       </c>
       <c r="I13">
@@ -6291,406 +6299,406 @@
         <f t="shared" si="6"/>
         <v>-0.91502306367624497</v>
       </c>
-      <c r="M13" s="2">
+      <c r="M13">
         <v>161859</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13">
         <v>4.6666670000000003</v>
       </c>
-      <c r="O13" s="2">
+      <c r="O13">
         <v>4.3636359999999996</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13">
         <v>4.9230770000000001</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13">
         <v>4.7692310000000004</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13">
         <v>5.7142860000000004</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13">
         <v>5.8333329999999997</v>
       </c>
-      <c r="T13" s="2" t="s">
+      <c r="T13" t="s">
         <v>131</v>
       </c>
-      <c r="U13" s="2" t="s">
+      <c r="U13" t="s">
         <v>132</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13">
         <v>4.67</v>
       </c>
-      <c r="W13" s="2">
+      <c r="W13">
         <v>4</v>
       </c>
-      <c r="X13" s="2">
+      <c r="X13">
         <v>4</v>
       </c>
-      <c r="Y13" s="2">
+      <c r="Y13">
         <v>4</v>
       </c>
-      <c r="Z13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="2">
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
         <v>6.67</v>
       </c>
-      <c r="AB13" s="2">
+      <c r="AB13">
         <v>5.67</v>
       </c>
-      <c r="AC13" s="2">
+      <c r="AC13">
         <v>5.63</v>
       </c>
-      <c r="AD13" s="2">
+      <c r="AD13">
         <v>5.17</v>
       </c>
-      <c r="AE13" s="2">
+      <c r="AE13">
         <v>5.8</v>
       </c>
-      <c r="AF13" s="2">
+      <c r="AF13">
         <v>19</v>
       </c>
-      <c r="AG13" s="2">
+      <c r="AG13">
         <v>2</v>
       </c>
-      <c r="AH13" s="2">
+      <c r="AH13">
         <v>12</v>
       </c>
-      <c r="AI13" s="2">
+      <c r="AI13">
         <v>4</v>
       </c>
-      <c r="AJ13" s="2">
-        <v>1</v>
-      </c>
-      <c r="AK13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AL13" s="2">
+      <c r="AJ13">
+        <v>1</v>
+      </c>
+      <c r="AK13">
+        <v>0</v>
+      </c>
+      <c r="AL13">
         <v>5</v>
       </c>
-      <c r="AM13" s="2">
+      <c r="AM13">
         <v>6</v>
       </c>
-      <c r="AN13" s="2">
-        <v>1</v>
-      </c>
-      <c r="AO13" s="2">
-        <v>1</v>
-      </c>
-      <c r="AP13" s="2">
+      <c r="AN13">
+        <v>1</v>
+      </c>
+      <c r="AO13">
+        <v>1</v>
+      </c>
+      <c r="AP13">
         <v>13</v>
       </c>
-      <c r="AQ13" s="2">
+      <c r="AQ13">
         <v>30</v>
       </c>
-      <c r="AR13" s="2">
+      <c r="AR13">
         <v>9</v>
       </c>
-      <c r="AS13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AT13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AU13" s="2">
+      <c r="AS13">
+        <v>0</v>
+      </c>
+      <c r="AT13">
+        <v>0</v>
+      </c>
+      <c r="AU13">
         <v>6</v>
       </c>
-      <c r="AV13" s="2">
+      <c r="AV13">
         <v>6</v>
       </c>
-      <c r="AW13" s="2">
+      <c r="AW13">
         <v>6</v>
       </c>
-      <c r="AX13" s="2">
+      <c r="AX13">
         <v>6</v>
       </c>
-      <c r="AZ13" s="2">
+      <c r="AZ13">
         <v>11</v>
       </c>
-      <c r="BA13" s="2">
+      <c r="BA13">
         <v>2.58</v>
       </c>
-      <c r="BC13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BD13" s="2">
+      <c r="BC13">
+        <v>0</v>
+      </c>
+      <c r="BD13">
         <v>3.43</v>
       </c>
-      <c r="BE13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BF13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BG13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BH13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BI13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BJ13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BK13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BL13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BM13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BN13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BO13" s="2">
+      <c r="BE13">
+        <v>0</v>
+      </c>
+      <c r="BF13">
+        <v>0</v>
+      </c>
+      <c r="BG13">
+        <v>0</v>
+      </c>
+      <c r="BH13">
+        <v>0</v>
+      </c>
+      <c r="BI13">
+        <v>0</v>
+      </c>
+      <c r="BJ13">
+        <v>0</v>
+      </c>
+      <c r="BK13">
+        <v>0</v>
+      </c>
+      <c r="BL13">
+        <v>0</v>
+      </c>
+      <c r="BM13">
+        <v>0</v>
+      </c>
+      <c r="BN13">
+        <v>0</v>
+      </c>
+      <c r="BO13">
         <v>20</v>
       </c>
-      <c r="BP13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BQ13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BR13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BS13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BT13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BU13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BV13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BW13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BX13" s="2">
+      <c r="BP13">
+        <v>0</v>
+      </c>
+      <c r="BQ13">
+        <v>0</v>
+      </c>
+      <c r="BR13">
+        <v>0</v>
+      </c>
+      <c r="BS13">
+        <v>0</v>
+      </c>
+      <c r="BT13">
+        <v>0</v>
+      </c>
+      <c r="BU13">
+        <v>0</v>
+      </c>
+      <c r="BV13">
+        <v>0</v>
+      </c>
+      <c r="BW13">
+        <v>0</v>
+      </c>
+      <c r="BX13">
         <v>8991</v>
       </c>
-      <c r="BY13" s="2">
-        <v>0</v>
-      </c>
-      <c r="BZ13" s="2">
-        <v>0</v>
-      </c>
-      <c r="CA13" s="2">
-        <v>0</v>
-      </c>
-      <c r="CB13" s="2">
-        <v>0</v>
-      </c>
-      <c r="CC13" s="2">
+      <c r="BY13">
+        <v>0</v>
+      </c>
+      <c r="BZ13">
+        <v>0</v>
+      </c>
+      <c r="CA13">
+        <v>0</v>
+      </c>
+      <c r="CB13">
+        <v>0</v>
+      </c>
+      <c r="CC13">
         <v>3.6</v>
       </c>
-      <c r="CD13" s="2">
+      <c r="CD13">
         <v>3.7</v>
       </c>
-      <c r="CE13" s="2">
+      <c r="CE13">
         <v>3.9</v>
       </c>
-      <c r="CF13" s="2">
+      <c r="CF13">
         <v>3.73</v>
       </c>
-      <c r="CG13" s="2">
+      <c r="CG13">
         <v>2.6666666666666599</v>
       </c>
-      <c r="CH13" s="2">
+      <c r="CH13">
         <v>3.3333333333333299</v>
       </c>
-      <c r="CI13" s="2">
+      <c r="CI13">
         <v>6</v>
       </c>
-      <c r="CJ13" s="2">
+      <c r="CJ13">
         <v>4</v>
       </c>
-      <c r="CK13" s="2">
+      <c r="CK13">
         <v>1.8</v>
       </c>
-      <c r="CL13" s="2">
-        <v>0</v>
-      </c>
-      <c r="CM13" s="2">
-        <v>0</v>
-      </c>
-      <c r="CN13" s="2">
+      <c r="CL13">
+        <v>0</v>
+      </c>
+      <c r="CM13">
+        <v>0</v>
+      </c>
+      <c r="CN13">
         <v>22</v>
       </c>
-      <c r="CO13" s="2">
+      <c r="CO13">
         <v>20</v>
       </c>
-      <c r="CP13" s="2">
+      <c r="CP13">
         <v>9</v>
       </c>
-      <c r="CQ13" s="2">
+      <c r="CQ13">
         <v>0.9</v>
       </c>
-      <c r="CR13" s="2">
+      <c r="CR13">
         <v>31</v>
       </c>
-      <c r="CS13" s="2">
+      <c r="CS13">
         <v>28</v>
       </c>
-      <c r="CT13" s="2">
+      <c r="CT13">
         <v>36</v>
       </c>
-      <c r="CU13" s="3">
+      <c r="CU13" s="1">
         <v>32</v>
       </c>
-      <c r="CV13" s="3">
+      <c r="CV13" s="1">
         <v>29</v>
       </c>
-      <c r="CW13" s="2">
+      <c r="CW13">
         <v>38</v>
       </c>
-      <c r="CX13" s="2">
+      <c r="CX13">
         <v>60</v>
       </c>
-      <c r="CY13" s="2">
+      <c r="CY13">
         <v>34</v>
       </c>
-      <c r="CZ13" s="2">
+      <c r="CZ13">
         <v>60</v>
       </c>
-      <c r="DA13" s="2">
+      <c r="DA13">
         <v>27</v>
       </c>
-      <c r="DB13" s="2">
+      <c r="DB13">
         <v>60</v>
       </c>
-      <c r="DC13" s="2">
-        <v>0</v>
-      </c>
-      <c r="DD13" s="2">
-        <v>0</v>
-      </c>
-      <c r="DE13" s="2">
+      <c r="DC13">
+        <v>0</v>
+      </c>
+      <c r="DD13">
+        <v>0</v>
+      </c>
+      <c r="DE13">
         <v>7</v>
       </c>
-      <c r="DF13" s="2">
-        <v>1</v>
-      </c>
-      <c r="DG13" s="2">
+      <c r="DF13">
+        <v>1</v>
+      </c>
+      <c r="DG13">
         <v>45106</v>
       </c>
-      <c r="DH13" s="2">
+      <c r="DH13">
         <v>21854</v>
       </c>
-      <c r="DI13" s="2">
+      <c r="DI13">
         <v>63.66</v>
       </c>
-      <c r="DJ13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DK13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DL13" s="2">
-        <v>0</v>
-      </c>
-      <c r="DM13" s="2">
-        <v>0</v>
-      </c>
-      <c r="DN13" s="2">
-        <v>1</v>
-      </c>
-      <c r="DO13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="DP13" s="2">
+      <c r="DJ13" t="s">
+        <v>133</v>
+      </c>
+      <c r="DK13" t="s">
+        <v>133</v>
+      </c>
+      <c r="DL13">
+        <v>0</v>
+      </c>
+      <c r="DM13">
+        <v>0</v>
+      </c>
+      <c r="DN13">
+        <v>1</v>
+      </c>
+      <c r="DO13" t="s">
+        <v>133</v>
+      </c>
+      <c r="DP13">
         <v>28</v>
       </c>
-      <c r="DQ13" s="2">
+      <c r="DQ13">
         <v>2.6111111111111001</v>
       </c>
-      <c r="DR13" s="2">
+      <c r="DR13">
         <v>12</v>
       </c>
-      <c r="DS13" s="2">
+      <c r="DS13">
         <v>999</v>
       </c>
-      <c r="DT13" s="2">
+      <c r="DT13">
         <v>7</v>
       </c>
-      <c r="DU13" s="2">
-        <v>1</v>
-      </c>
-      <c r="DV13" s="2">
+      <c r="DU13">
+        <v>1</v>
+      </c>
+      <c r="DV13">
         <v>999</v>
       </c>
-      <c r="DW13" s="2">
+      <c r="DW13">
         <v>10</v>
       </c>
-      <c r="DY13" s="2">
+      <c r="DY13">
         <v>6</v>
       </c>
-      <c r="DZ13" s="2">
+      <c r="DZ13">
         <v>3</v>
       </c>
-      <c r="EA13" s="2">
+      <c r="EA13">
         <v>8</v>
       </c>
-      <c r="EB13" s="2">
+      <c r="EB13">
         <v>6</v>
       </c>
-      <c r="EC13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ED13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EE13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EF13" s="2">
+      <c r="EC13" t="s">
+        <v>133</v>
+      </c>
+      <c r="ED13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EE13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EF13">
         <v>2</v>
       </c>
-      <c r="EG13" s="2">
+      <c r="EG13">
         <v>11793</v>
       </c>
-      <c r="EH13" s="2">
+      <c r="EH13">
         <v>8</v>
       </c>
-      <c r="EI13" s="2">
-        <v>1</v>
-      </c>
-      <c r="EJ13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EK13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EL13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EM13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EN13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EO13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EP13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="EQ13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="ER13" s="2">
-        <v>0</v>
-      </c>
-      <c r="ES13" s="2" t="s">
+      <c r="EI13">
+        <v>1</v>
+      </c>
+      <c r="EJ13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EK13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EL13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EM13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EN13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EO13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EP13" t="s">
+        <v>133</v>
+      </c>
+      <c r="EQ13" t="s">
+        <v>133</v>
+      </c>
+      <c r="ER13">
+        <v>0</v>
+      </c>
+      <c r="ES13" t="s">
         <v>133</v>
       </c>
     </row>
@@ -27284,6 +27292,24 @@
       <c r="H60">
         <f t="shared" ref="H60" si="8">AVERAGE(H2:H59)</f>
         <v>4.4015151515151478</v>
+      </c>
+    </row>
+    <row r="61" spans="1:149" x14ac:dyDescent="0.2">
+      <c r="B61">
+        <f>STDEV(B2:B59)</f>
+        <v>16.840751776187894</v>
+      </c>
+    </row>
+    <row r="62" spans="1:149" x14ac:dyDescent="0.2">
+      <c r="B62">
+        <f>MIN(B2:B59)</f>
+        <v>21.43</v>
+      </c>
+    </row>
+    <row r="63" spans="1:149" x14ac:dyDescent="0.2">
+      <c r="B63">
+        <f>MAX(B2:B59)</f>
+        <v>73.400000000000006</v>
       </c>
     </row>
   </sheetData>
@@ -27363,7 +27389,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>10486</v>
       </c>
       <c r="B7">
@@ -27396,7 +27422,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10">
         <v>10572</v>
       </c>
       <c r="B10">
@@ -27429,7 +27455,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13">
         <v>10585</v>
       </c>
       <c r="B13">
@@ -28058,7 +28084,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>10486</v>
       </c>
       <c r="B7">
@@ -28109,7 +28135,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10">
         <v>10572</v>
       </c>
       <c r="B10">
@@ -28160,7 +28186,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13">
         <v>10585</v>
       </c>
       <c r="B13">
@@ -29071,7 +29097,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>10486</v>
       </c>
       <c r="B7">
@@ -29122,7 +29148,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10">
         <v>10572</v>
       </c>
       <c r="B10">
@@ -29173,7 +29199,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13">
         <v>10585</v>
       </c>
       <c r="B13">
@@ -30156,7 +30182,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>10486</v>
       </c>
       <c r="B7">
@@ -30243,7 +30269,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10">
         <v>10572</v>
       </c>
       <c r="B10">
@@ -30330,7 +30356,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13">
         <v>10585</v>
       </c>
       <c r="B13">
@@ -31690,6 +31716,1035 @@
       </c>
       <c r="I59">
         <v>97.997010230021687</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{108F8D1E-1458-834C-82BC-7E525D9AD5DA}">
+  <dimension ref="A1:G56"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>10369</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>-10.256181818181812</v>
+      </c>
+      <c r="D2">
+        <v>9.8484848484852172E-2</v>
+      </c>
+      <c r="E2">
+        <f>C2*D2</f>
+        <v>-1.0100785123967313</v>
+      </c>
+      <c r="G2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>10402</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>-6.2661818181818134</v>
+      </c>
+      <c r="D3">
+        <v>-1.1515151515151478</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E56" si="0">C3*D3</f>
+        <v>7.2156033057850957</v>
+      </c>
+      <c r="G3">
+        <v>10486</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>10418</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>26.433818181818189</v>
+      </c>
+      <c r="D4">
+        <v>0.34848484848485217</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>9.2117851239670419</v>
+      </c>
+      <c r="G4">
+        <v>10572</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>10462</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>19.833818181818188</v>
+      </c>
+      <c r="D5">
+        <v>-0.15151515151514783</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>-3.0051239669420764</v>
+      </c>
+      <c r="G5">
+        <v>10585</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>10478</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>-14.306181818181813</v>
+      </c>
+      <c r="D6">
+        <v>9.8484848484852172E-2</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>-1.4089421487603828</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>10529</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>25.593818181818186</v>
+      </c>
+      <c r="D7">
+        <v>-0.90151515151514783</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>-23.073214876032967</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>10541</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>26.953818181818185</v>
+      </c>
+      <c r="D8">
+        <v>-0.8181818181818179</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>-22.053123966942145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>10581</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>5.82381818181819</v>
+      </c>
+      <c r="D9">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>3.4854669421487867</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>10584</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>7.4338181818181894</v>
+      </c>
+      <c r="D10">
+        <v>-0.90151515151514783</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>-6.7016997245178862</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10589</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>-7.3361818181818137</v>
+      </c>
+      <c r="D11">
+        <v>-0.8181818181818179</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>6.0023305785123906</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>10590</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>14.193818181818187</v>
+      </c>
+      <c r="D12">
+        <v>-0.23484848484848797</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>-3.3333966942149216</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>10596</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>-14.936181818181812</v>
+      </c>
+      <c r="D13">
+        <v>-6.8181818181817455E-2</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>1.01837603305784</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>10603</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>27.013818181818188</v>
+      </c>
+      <c r="D14">
+        <v>-0.23484848484848797</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>-6.3441542699725373</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>10606</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>-19.806181818181813</v>
+      </c>
+      <c r="D15">
+        <v>-0.48484848484848797</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>9.6029972451791217</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>10608</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>-13.136181818181811</v>
+      </c>
+      <c r="D16">
+        <v>-0.48484848484848797</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>6.3690578512397069</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>10617</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>31.193818181818195</v>
+      </c>
+      <c r="D17">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>18.669027548209488</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>10636</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>-15.396181818181812</v>
+      </c>
+      <c r="D18">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>-9.2143815426997779</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>10638</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>29.623818181818187</v>
+      </c>
+      <c r="D19">
+        <v>-0.484848484848448</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>-14.363063360880453</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>10640</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>-10.476181818181811</v>
+      </c>
+      <c r="D20">
+        <v>0.43181818181815235</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>-4.5238057851236553</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>10641</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>2.4738181818181886</v>
+      </c>
+      <c r="D21">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>1.480542699724531</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>10642</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>-10.306181818181813</v>
+      </c>
+      <c r="D22">
+        <v>-1.6515151515151478</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>17.020815426997199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>10644</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>27.203818181818185</v>
+      </c>
+      <c r="D23">
+        <v>-0.31818181818181746</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="0"/>
+        <v>-8.6557603305784934</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>10647</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>-17.616181818181811</v>
+      </c>
+      <c r="D24">
+        <v>0.18181818181815235</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="0"/>
+        <v>-3.20294214875981</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>10649</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>21.593818181818186</v>
+      </c>
+      <c r="D25">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="0"/>
+        <v>12.923573002754903</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>10652</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>27.843818181818186</v>
+      </c>
+      <c r="D26">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>16.664103305785229</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>10656</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>-20.776181818181811</v>
+      </c>
+      <c r="D27">
+        <v>-0.98484848484848797</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="0"/>
+        <v>20.46139118457306</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>10657</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>16.773818181818186</v>
+      </c>
+      <c r="D28">
+        <v>-0.65151515151514783</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="0"/>
+        <v>-10.928396694214817</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>10659</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29">
+        <v>20.183818181818189</v>
+      </c>
+      <c r="D29">
+        <v>-0.5681818181818179</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="0"/>
+        <v>-11.468078512396692</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>10663</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>-20.136181818181811</v>
+      </c>
+      <c r="D30">
+        <v>0.26515151515151203</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="0"/>
+        <v>-5.3391391184572354</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>10673</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31">
+        <v>6.3938181818181903</v>
+      </c>
+      <c r="D31">
+        <v>-0.23484848484848797</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="0"/>
+        <v>-1.5015785123967162</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>10674</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32">
+        <v>-9.0061818181818083</v>
+      </c>
+      <c r="D32">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="0"/>
+        <v>-5.3900633608815696</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>10677</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>-8.8361818181818137</v>
+      </c>
+      <c r="D33">
+        <v>9.8484848484852172E-2</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="0"/>
+        <v>-0.87023002754824152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>10685</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34">
+        <v>-7.7761818181818114</v>
+      </c>
+      <c r="D34">
+        <v>1.515151515151512</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="0"/>
+        <v>-11.782093663911811</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>10691</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35">
+        <v>16.063818181818192</v>
+      </c>
+      <c r="D35">
+        <v>-1.984848484848488</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="0"/>
+        <v>-31.884245179063431</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>10700</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36">
+        <v>-18.596181818181812</v>
+      </c>
+      <c r="D36">
+        <v>0.84848484848485217</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="0"/>
+        <v>-15.778578512396757</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>10701</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37">
+        <v>-15.186181818181812</v>
+      </c>
+      <c r="D37">
+        <v>-1.8181818181818179</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="0"/>
+        <v>27.611239669421472</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>10718</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38">
+        <v>-13.90618181818181</v>
+      </c>
+      <c r="D38">
+        <v>0.59848484848485217</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="0"/>
+        <v>-8.3226391184573476</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>10720</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>-8.7661818181818134</v>
+      </c>
+      <c r="D39">
+        <v>1.5984848484848522</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="0"/>
+        <v>-14.012608815427022</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>10723</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40">
+        <v>-20.506181818181812</v>
+      </c>
+      <c r="D40">
+        <v>-0.48484848484848797</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="0"/>
+        <v>9.9423911845730633</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>10741</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41">
+        <v>-5.2761818181818114</v>
+      </c>
+      <c r="D41">
+        <v>-6.8181818181817455E-2</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="0"/>
+        <v>0.35973966942148333</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>10748</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42">
+        <v>-8.906181818181814</v>
+      </c>
+      <c r="D42">
+        <v>-0.48484848484848797</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="0"/>
+        <v>4.3181487603306046</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>10767</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43">
+        <v>-16.69618181818181</v>
+      </c>
+      <c r="D43">
+        <v>0.43181818181818254</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="0"/>
+        <v>-7.2097148760330665</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>10774</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44">
+        <v>3.7938181818181889</v>
+      </c>
+      <c r="D44">
+        <v>1.9318181818181825</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="0"/>
+        <v>7.3289669421487771</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>10777</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45">
+        <v>-3.8461818181818117</v>
+      </c>
+      <c r="D45">
+        <v>-0.73484848484848797</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="0"/>
+        <v>2.826360881542707</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>10781</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46">
+        <v>-4.67618181818181</v>
+      </c>
+      <c r="D46">
+        <v>1.765151515151512</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="0"/>
+        <v>-8.2541694214875747</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>10783</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47">
+        <v>8.9738181818181886</v>
+      </c>
+      <c r="D47">
+        <v>1.265151515151512</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="0"/>
+        <v>11.353239669421468</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>10785</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48">
+        <v>19.023818181818186</v>
+      </c>
+      <c r="D48">
+        <v>-1.6515151515151478</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="0"/>
+        <v>-31.418123966942083</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>10794</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49">
+        <v>-2.5161818181818134</v>
+      </c>
+      <c r="D49">
+        <v>0.26515151515151203</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="0"/>
+        <v>-0.66716942148759417</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>10800</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50">
+        <v>-15.35618181818181</v>
+      </c>
+      <c r="D50">
+        <v>1.515151515151512</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="0"/>
+        <v>-23.266942148760268</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>10801</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51">
+        <v>-7.67618181818181</v>
+      </c>
+      <c r="D51">
+        <v>-1.8181818181818179</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="0"/>
+        <v>13.956694214876016</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>10802</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52">
+        <v>0.48381818181818659</v>
+      </c>
+      <c r="D52">
+        <v>2.015151515151512</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="0"/>
+        <v>0.97496694214876845</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>10803</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53">
+        <v>-20.546181818181811</v>
+      </c>
+      <c r="D53">
+        <v>-0.23484848484848797</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="0"/>
+        <v>4.82523966942155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>10804</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54">
+        <v>-16.706181818181811</v>
+      </c>
+      <c r="D54">
+        <v>-0.15151515151514783</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="0"/>
+        <v>2.5312396694214248</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>10806</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55">
+        <v>-15.216181818181813</v>
+      </c>
+      <c r="D55">
+        <v>-1.484848484848488</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="0"/>
+        <v>22.593724517906374</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>10807</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56">
+        <v>15.843818181818186</v>
+      </c>
+      <c r="D56">
+        <v>2.5984848484848522</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="0"/>
+        <v>41.169921487603375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>